<commit_message>
Use literal values instead of formulas for Cost sheet totals
Some spreadsheet viewers don't recalculate formulas on open, leaving
subtotals/grand total blank or zero. Write computed numeric values so
totals always display.

https://claude.ai/code/session_01NtYwhcGqR4ohrSJiJsSbvP
</commit_message>
<xml_diff>
--- a/Family_Holiday_Itinerary_2026.xlsx
+++ b/Family_Holiday_Itinerary_2026.xlsx
@@ -1949,9 +1949,8 @@
           <t>Flights subtotal</t>
         </is>
       </c>
-      <c r="C11" s="17">
-        <f>SUM(C6:C10)</f>
-        <v/>
+      <c r="C11" s="17" t="n">
+        <v>28000</v>
       </c>
     </row>
     <row r="13">
@@ -2046,9 +2045,8 @@
           <t>Accommodation subtotal</t>
         </is>
       </c>
-      <c r="C19" s="17">
-        <f>SUM(C15:C18)</f>
-        <v/>
+      <c r="C19" s="17" t="n">
+        <v>6430</v>
       </c>
     </row>
     <row r="21">
@@ -2058,9 +2056,8 @@
           <t>GRAND TOTAL (flights + accommodation)</t>
         </is>
       </c>
-      <c r="C21" s="20">
-        <f>C11+C19</f>
-        <v/>
+      <c r="C21" s="20" t="n">
+        <v>34430</v>
       </c>
     </row>
     <row r="23">

</xml_diff>